<commit_message>
Added LicenseDecoder and some Vest types
</commit_message>
<xml_diff>
--- a/References/All things about vest.xlsx
+++ b/References/All things about vest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shdxz\Desktop\Vest\References\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7C8F4D1-FB22-4B92-A3FD-1F63C9786DAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F77CCE1-1AC0-4E2E-967B-63CA470CD6C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="17445" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="13763" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Types" sheetId="1" r:id="rId1"/>
@@ -177,10 +177,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>VEST_ANYARRAY</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>VEST_DATA</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -190,6 +186,10 @@
   </si>
   <si>
     <t>VEST_SET</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VEST_LIST</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -724,35 +724,35 @@
     </row>
     <row r="15" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>31</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>32</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Adding new features in classes
</commit_message>
<xml_diff>
--- a/References/All things about vest.xlsx
+++ b/References/All things about vest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shdxz\Desktop\Vest\References\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F77CCE1-1AC0-4E2E-967B-63CA470CD6C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{161B5E0D-87B5-49AF-ACBD-C6311045C8BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="13763" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-60" yWindow="-60" windowWidth="21720" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Types" sheetId="1" r:id="rId1"/>
@@ -220,7 +220,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -236,6 +236,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -267,7 +279,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -279,6 +291,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -591,7 +609,7 @@
       </c>
     </row>
     <row r="3" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="5" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -602,7 +620,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -613,7 +631,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -624,7 +642,7 @@
       </c>
     </row>
     <row r="6" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="5" t="s">
         <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -635,7 +653,7 @@
       </c>
     </row>
     <row r="7" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="6" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">

</xml_diff>

<commit_message>
Modified .gitignore and did some code
</commit_message>
<xml_diff>
--- a/References/All things about vest.xlsx
+++ b/References/All things about vest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shdxz\Desktop\Vest\References\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F77CCE1-1AC0-4E2E-967B-63CA470CD6C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6EF35FA-4B74-4E8F-9127-EC0E61712EFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="13763" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Types" sheetId="1" r:id="rId1"/>
@@ -220,7 +220,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -236,6 +236,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -267,7 +273,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -279,6 +285,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -591,7 +600,7 @@
       </c>
     </row>
     <row r="3" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="5" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -602,7 +611,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -613,7 +622,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -624,7 +633,7 @@
       </c>
     </row>
     <row r="6" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="5" t="s">
         <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -635,7 +644,7 @@
       </c>
     </row>
     <row r="7" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -646,7 +655,7 @@
       </c>
     </row>
     <row r="8" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -657,7 +666,7 @@
       </c>
     </row>
     <row r="9" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="5" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -668,7 +677,7 @@
       </c>
     </row>
     <row r="10" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">

</xml_diff>